<commit_message>
actualiza acumulados 22/06/2026 10:19
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO-LUCILA-RUBIO-DE-LAVERDE-(IED)-701_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO-LUCILA-RUBIO-DE-LAVERDE-(IED)-701_CALIFICADO.xlsx
@@ -8385,11 +8385,7 @@
           <t>KAROL SOFIA GUZMAN LOPEZ</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>1030648404</t>
-        </is>
-      </c>
+      <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="n">
         <v>7</v>
       </c>
@@ -8638,11 +8634,7 @@
           <t>KAROL SOFIA GUZMAN LOPEZ</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>1030648404</t>
-        </is>
-      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="2" t="n">
         <v>7</v>
       </c>

</xml_diff>